<commit_message>
docs: new example file without extra columns
</commit_message>
<xml_diff>
--- a/free-all-fta-example.xlsx
+++ b/free-all-fta-example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raphaelbaroni/code/infrabel/free-all-fta/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ARM8001\Downloads\free-all-fta-main\free-all-fta-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8DECAE6-58A1-B044-A6D3-BF3F7A017550}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F80D66D1-0FBE-4DCA-9FB1-C7DA5FF4F723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25600" yWindow="0" windowWidth="25600" windowHeight="27000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32340" yWindow="1755" windowWidth="21600" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="events" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
     <definedName name="GATE_TYPES">lists!$B$2:$B$20</definedName>
     <definedName name="maintenanceInterval">specificData!$C$2</definedName>
   </definedNames>
-  <calcPr calcId="191029" forceFullCalc="1"/>
+  <calcPr calcId="191029" iterateDelta="1E-4" forceFullCalc="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="198">
   <si>
     <t>id</t>
   </si>
@@ -627,6 +627,42 @@
   </si>
   <si>
     <t>MAINT_INT</t>
+  </si>
+  <si>
+    <t>Dangerous loss of UL1 when UL1 detected faulty</t>
+  </si>
+  <si>
+    <t>DANGEROUS_LOSS_ALARM1_WHEN_UL1_DETECTED_FAULTY</t>
+  </si>
+  <si>
+    <t>DANGEROUS_LOSS_ALARM2_WHEN_UL2_DETECTED_FAULTY</t>
+  </si>
+  <si>
+    <t>Dangerous loss of UL2 when UL2 detected faulty</t>
+  </si>
+  <si>
+    <t>DANGEROUS_LOSS_ALARM1_WHEN_UL1_DETECTED_FAULTY - Dangerous loss of UL1 when UL1 detected faulty</t>
+  </si>
+  <si>
+    <t>DANGEROUS_LOSS_ALARM2_WHEN_UL2_DETECTED_FAULTY - Dangerous loss of UL2 when UL2 detected faulty</t>
+  </si>
+  <si>
+    <t>UL1_NOT_DETECTED_FAULTY_BY_ITSELF</t>
+  </si>
+  <si>
+    <t>UL2_NOT_DETECTED_FAULTY_BY_ITSELF</t>
+  </si>
+  <si>
+    <t>UL2 not detected faulty by itself and no opening of internal circuit</t>
+  </si>
+  <si>
+    <t>UL1 not detected faulty by itself and no opening of internal circuit</t>
+  </si>
+  <si>
+    <t>UL1_NOT_DETECTED_FAULTY_BY_ITSELF - UL1 not detected faulty by itself and no opening of internal circuit</t>
+  </si>
+  <si>
+    <t>UL2_NOT_DETECTED_FAULTY_BY_ITSELF - UL2 not detected faulty by itself and no opening of internal circuit</t>
   </si>
 </sst>
 </file>
@@ -782,6 +818,9 @@
   </cellStyles>
   <dxfs count="56">
     <dxf>
+      <numFmt numFmtId="15" formatCode="0.00E+00"/>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <strike val="0"/>
@@ -970,9 +1009,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="15" formatCode="0.00E+00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="15" formatCode="0.00E+00"/>
@@ -1011,8 +1047,8 @@
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="probability"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="intensity"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="comment"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Allocated value" dataDxfId="54"/>
-    <tableColumn id="13" xr3:uid="{BF1D39E4-2844-B149-99CC-BAD2D8712528}" name="Formula" dataDxfId="53"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Allocated value" dataDxfId="0"/>
+    <tableColumn id="13" xr3:uid="{BF1D39E4-2844-B149-99CC-BAD2D8712528}" name="Formula" dataDxfId="54"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="appearance"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1020,26 +1056,26 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tbl_gates" displayName="tbl_gates" ref="A1:I14" dataDxfId="52">
-  <autoFilter ref="A1:I14" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tbl_gates" displayName="tbl_gates" ref="A1:I18" dataDxfId="53">
+  <autoFilter ref="A1:I18" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="id" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="label" dataDxfId="50"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="comment" dataDxfId="49"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="Formula" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="is_paged" dataDxfId="47"/>
-    <tableColumn id="11" xr3:uid="{8333B313-5288-47B1-81E6-DDC72BDF0941}" name="safety target" dataDxfId="46"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="calculated frequency" dataDxfId="45"/>
-    <tableColumn id="14" xr3:uid="{61DA1A62-3985-1D44-AAAE-28E2F281A6DA}" name="calculated mean repair time" dataDxfId="44"/>
-    <tableColumn id="12" xr3:uid="{07A48EEF-A119-490F-93B9-C6CF45F7B687}" name="differences" dataDxfId="43"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="id" dataDxfId="52"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="label" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="comment" dataDxfId="50"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="Formula" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="is_paged" dataDxfId="48"/>
+    <tableColumn id="11" xr3:uid="{8333B313-5288-47B1-81E6-DDC72BDF0941}" name="safety target" dataDxfId="47"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="calculated frequency" dataDxfId="46"/>
+    <tableColumn id="14" xr3:uid="{61DA1A62-3985-1D44-AAAE-28E2F281A6DA}" name="calculated mean repair time" dataDxfId="45"/>
+    <tableColumn id="12" xr3:uid="{07A48EEF-A119-490F-93B9-C6CF45F7B687}" name="differences" dataDxfId="44"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A47E647F-585F-AE4C-A62C-2BA782B5E934}" name="tbl_tree" displayName="tbl_tree" ref="A1:AN101" totalsRowShown="0" headerRowDxfId="42" dataDxfId="41">
-  <autoFilter ref="A1:AN101" xr:uid="{A47E647F-585F-AE4C-A62C-2BA782B5E934}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A47E647F-585F-AE4C-A62C-2BA782B5E934}" name="tbl_tree" displayName="tbl_tree" ref="A1:AN107" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
+  <autoFilter ref="A1:AN107" xr:uid="{A47E647F-585F-AE4C-A62C-2BA782B5E934}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1082,53 +1118,53 @@
     <filterColumn colId="39" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="40">
-    <tableColumn id="1" xr3:uid="{401229BE-F777-B648-AE80-B807F1E2DBFC}" name="L01_ID" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{31C3F4C1-452D-7147-B96D-B11AA9C79643}" name="L01_TYPE" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{5B218165-B150-EC43-BCAD-802C524E86D9}" name="L02_ID" dataDxfId="38"/>
-    <tableColumn id="4" xr3:uid="{9573DEBC-53D3-2143-984B-92A463E9E60D}" name="L02_TYPE" dataDxfId="37"/>
-    <tableColumn id="5" xr3:uid="{13692F6C-6DE1-9D4C-8577-E574E0A8EB6B}" name="L03_ID" dataDxfId="36"/>
-    <tableColumn id="6" xr3:uid="{426976C6-C7E5-D04E-9DBB-1C557388B7C9}" name="L03_TYPE" dataDxfId="35"/>
-    <tableColumn id="7" xr3:uid="{A915D8C9-CEFE-244F-B433-F660D6E50C7C}" name="L04_ID" dataDxfId="34"/>
-    <tableColumn id="8" xr3:uid="{65197F2C-EF25-2E46-90B6-895E98CFD7C0}" name="L04_TYPE" dataDxfId="33"/>
-    <tableColumn id="9" xr3:uid="{E910C4D6-3B54-A648-BFA1-FC01EA7A2A55}" name="L05_ID" dataDxfId="32"/>
-    <tableColumn id="10" xr3:uid="{D2B03439-4D4E-CD47-97DE-E0B3A5FDB1F1}" name="L05_TYPE" dataDxfId="31"/>
-    <tableColumn id="11" xr3:uid="{74C0B85A-B832-8741-A2D9-08DC2F4879AA}" name="L06_ID" dataDxfId="30"/>
-    <tableColumn id="12" xr3:uid="{B92EBD9D-4A24-DA4A-88C4-0A81D07D8086}" name="L06_TYPE" dataDxfId="29"/>
-    <tableColumn id="13" xr3:uid="{016DA4C7-8215-B641-AD4D-C1D0DF327F77}" name="L07_ID" dataDxfId="28"/>
-    <tableColumn id="14" xr3:uid="{637CBFF4-5BB8-FF42-9B02-7A1987F94AC3}" name="L07_TYPE" dataDxfId="27"/>
-    <tableColumn id="15" xr3:uid="{C137B6B5-D13D-1F4A-BA2C-1A3E8B920758}" name="L08_ID" dataDxfId="26"/>
-    <tableColumn id="16" xr3:uid="{464C3E7E-32D0-E241-9877-754248AC55C7}" name="L08_TYPE" dataDxfId="25"/>
-    <tableColumn id="17" xr3:uid="{BA46960E-541C-E145-825C-59128A6C743F}" name="L09_ID" dataDxfId="24"/>
-    <tableColumn id="18" xr3:uid="{E89CC4AD-95EB-014D-8DBE-F436EF55466C}" name="L09_TYPE" dataDxfId="23"/>
-    <tableColumn id="19" xr3:uid="{3FD6C545-44B8-3842-A759-88777B042795}" name="L10_ID" dataDxfId="22"/>
-    <tableColumn id="20" xr3:uid="{49356C37-1B14-B149-A924-F584A8E8E673}" name="L10_TYPE" dataDxfId="21"/>
-    <tableColumn id="21" xr3:uid="{7C5FFA16-5A9A-1841-9030-4DA307AA50F0}" name="L11_ID" dataDxfId="20"/>
-    <tableColumn id="22" xr3:uid="{8A93973C-3CC4-8A40-B55F-100EFCE8D7F7}" name="L11_TYPE" dataDxfId="19"/>
-    <tableColumn id="23" xr3:uid="{DD76C8F8-6BA5-C845-A77A-5D1AA0A77864}" name="L12_ID" dataDxfId="18"/>
-    <tableColumn id="24" xr3:uid="{8AC64CA4-93F0-2141-BD50-E4D9DD9C9024}" name="L12_TYPE" dataDxfId="17"/>
-    <tableColumn id="25" xr3:uid="{550DF0A2-6801-F749-88B2-A7A835E56182}" name="L13_ID" dataDxfId="16"/>
-    <tableColumn id="26" xr3:uid="{4C3EE3EC-7A40-A841-BAD0-48E3C334E8D9}" name="L13_TYPE" dataDxfId="15"/>
-    <tableColumn id="27" xr3:uid="{A6E49830-6955-B84A-B566-FF0B78EB30E6}" name="L14_ID" dataDxfId="14"/>
-    <tableColumn id="28" xr3:uid="{3F3D56A9-52B2-004D-9499-9ACD30BA203A}" name="L14_TYPE" dataDxfId="13"/>
-    <tableColumn id="29" xr3:uid="{DCA847E6-73C7-AD4A-960B-D591D0E6C11A}" name="L15_ID" dataDxfId="12"/>
-    <tableColumn id="30" xr3:uid="{543887BE-4EF7-6B47-B927-990C4BE01825}" name="L15_TYPE" dataDxfId="11"/>
-    <tableColumn id="31" xr3:uid="{10C180E8-3949-1D45-9E94-282515BEF145}" name="L16_ID" dataDxfId="10"/>
-    <tableColumn id="32" xr3:uid="{B7EBB1B1-1735-5B47-B9CC-948159228310}" name="L16_TYPE" dataDxfId="9"/>
-    <tableColumn id="33" xr3:uid="{7206A6CF-69C5-FC4E-A9E8-264B0D1E4726}" name="L17_ID" dataDxfId="8"/>
-    <tableColumn id="34" xr3:uid="{07AD8DCD-4D45-EA40-A9A2-2688AB7F6684}" name="L17_TYPE" dataDxfId="7"/>
-    <tableColumn id="35" xr3:uid="{4E7AF7BF-AA4E-3F47-B180-C2D529E62147}" name="L18_ID" dataDxfId="6"/>
-    <tableColumn id="36" xr3:uid="{017442D9-AE75-0A48-94BC-7049EBAFE4FE}" name="L18_TYPE" dataDxfId="5"/>
-    <tableColumn id="37" xr3:uid="{9DBC7FA0-99D9-CE41-8900-053581244511}" name="L19_ID" dataDxfId="4"/>
-    <tableColumn id="38" xr3:uid="{C3EA22FE-AE6C-C442-B5A7-EDEB4B3ED9F3}" name="L19_TYPE" dataDxfId="3"/>
-    <tableColumn id="39" xr3:uid="{78974802-75A4-5C43-8DF9-40DF43417107}" name="L20_ID" dataDxfId="2"/>
-    <tableColumn id="40" xr3:uid="{832CCD5E-4CF4-6448-BD02-1BB12881934A}" name="L20_TYPE" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{401229BE-F777-B648-AE80-B807F1E2DBFC}" name="L01_ID" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{31C3F4C1-452D-7147-B96D-B11AA9C79643}" name="L01_TYPE" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{5B218165-B150-EC43-BCAD-802C524E86D9}" name="L02_ID" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{9573DEBC-53D3-2143-984B-92A463E9E60D}" name="L02_TYPE" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{13692F6C-6DE1-9D4C-8577-E574E0A8EB6B}" name="L03_ID" dataDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{426976C6-C7E5-D04E-9DBB-1C557388B7C9}" name="L03_TYPE" dataDxfId="36"/>
+    <tableColumn id="7" xr3:uid="{A915D8C9-CEFE-244F-B433-F660D6E50C7C}" name="L04_ID" dataDxfId="35"/>
+    <tableColumn id="8" xr3:uid="{65197F2C-EF25-2E46-90B6-895E98CFD7C0}" name="L04_TYPE" dataDxfId="34"/>
+    <tableColumn id="9" xr3:uid="{E910C4D6-3B54-A648-BFA1-FC01EA7A2A55}" name="L05_ID" dataDxfId="33"/>
+    <tableColumn id="10" xr3:uid="{D2B03439-4D4E-CD47-97DE-E0B3A5FDB1F1}" name="L05_TYPE" dataDxfId="32"/>
+    <tableColumn id="11" xr3:uid="{74C0B85A-B832-8741-A2D9-08DC2F4879AA}" name="L06_ID" dataDxfId="31"/>
+    <tableColumn id="12" xr3:uid="{B92EBD9D-4A24-DA4A-88C4-0A81D07D8086}" name="L06_TYPE" dataDxfId="30"/>
+    <tableColumn id="13" xr3:uid="{016DA4C7-8215-B641-AD4D-C1D0DF327F77}" name="L07_ID" dataDxfId="29"/>
+    <tableColumn id="14" xr3:uid="{637CBFF4-5BB8-FF42-9B02-7A1987F94AC3}" name="L07_TYPE" dataDxfId="28"/>
+    <tableColumn id="15" xr3:uid="{C137B6B5-D13D-1F4A-BA2C-1A3E8B920758}" name="L08_ID" dataDxfId="27"/>
+    <tableColumn id="16" xr3:uid="{464C3E7E-32D0-E241-9877-754248AC55C7}" name="L08_TYPE" dataDxfId="26"/>
+    <tableColumn id="17" xr3:uid="{BA46960E-541C-E145-825C-59128A6C743F}" name="L09_ID" dataDxfId="25"/>
+    <tableColumn id="18" xr3:uid="{E89CC4AD-95EB-014D-8DBE-F436EF55466C}" name="L09_TYPE" dataDxfId="24"/>
+    <tableColumn id="19" xr3:uid="{3FD6C545-44B8-3842-A759-88777B042795}" name="L10_ID" dataDxfId="23"/>
+    <tableColumn id="20" xr3:uid="{49356C37-1B14-B149-A924-F584A8E8E673}" name="L10_TYPE" dataDxfId="22"/>
+    <tableColumn id="21" xr3:uid="{7C5FFA16-5A9A-1841-9030-4DA307AA50F0}" name="L11_ID" dataDxfId="21"/>
+    <tableColumn id="22" xr3:uid="{8A93973C-3CC4-8A40-B55F-100EFCE8D7F7}" name="L11_TYPE" dataDxfId="20"/>
+    <tableColumn id="23" xr3:uid="{DD76C8F8-6BA5-C845-A77A-5D1AA0A77864}" name="L12_ID" dataDxfId="19"/>
+    <tableColumn id="24" xr3:uid="{8AC64CA4-93F0-2141-BD50-E4D9DD9C9024}" name="L12_TYPE" dataDxfId="18"/>
+    <tableColumn id="25" xr3:uid="{550DF0A2-6801-F749-88B2-A7A835E56182}" name="L13_ID" dataDxfId="17"/>
+    <tableColumn id="26" xr3:uid="{4C3EE3EC-7A40-A841-BAD0-48E3C334E8D9}" name="L13_TYPE" dataDxfId="16"/>
+    <tableColumn id="27" xr3:uid="{A6E49830-6955-B84A-B566-FF0B78EB30E6}" name="L14_ID" dataDxfId="15"/>
+    <tableColumn id="28" xr3:uid="{3F3D56A9-52B2-004D-9499-9ACD30BA203A}" name="L14_TYPE" dataDxfId="14"/>
+    <tableColumn id="29" xr3:uid="{DCA847E6-73C7-AD4A-960B-D591D0E6C11A}" name="L15_ID" dataDxfId="13"/>
+    <tableColumn id="30" xr3:uid="{543887BE-4EF7-6B47-B927-990C4BE01825}" name="L15_TYPE" dataDxfId="12"/>
+    <tableColumn id="31" xr3:uid="{10C180E8-3949-1D45-9E94-282515BEF145}" name="L16_ID" dataDxfId="11"/>
+    <tableColumn id="32" xr3:uid="{B7EBB1B1-1735-5B47-B9CC-948159228310}" name="L16_TYPE" dataDxfId="10"/>
+    <tableColumn id="33" xr3:uid="{7206A6CF-69C5-FC4E-A9E8-264B0D1E4726}" name="L17_ID" dataDxfId="9"/>
+    <tableColumn id="34" xr3:uid="{07AD8DCD-4D45-EA40-A9A2-2688AB7F6684}" name="L17_TYPE" dataDxfId="8"/>
+    <tableColumn id="35" xr3:uid="{4E7AF7BF-AA4E-3F47-B180-C2D529E62147}" name="L18_ID" dataDxfId="7"/>
+    <tableColumn id="36" xr3:uid="{017442D9-AE75-0A48-94BC-7049EBAFE4FE}" name="L18_TYPE" dataDxfId="6"/>
+    <tableColumn id="37" xr3:uid="{9DBC7FA0-99D9-CE41-8900-053581244511}" name="L19_ID" dataDxfId="5"/>
+    <tableColumn id="38" xr3:uid="{C3EA22FE-AE6C-C442-B5A7-EDEB4B3ED9F3}" name="L19_TYPE" dataDxfId="4"/>
+    <tableColumn id="39" xr3:uid="{78974802-75A4-5C43-8DF9-40DF43417107}" name="L20_ID" dataDxfId="3"/>
+    <tableColumn id="40" xr3:uid="{832CCD5E-4CF4-6448-BD02-1BB12881934A}" name="L20_TYPE" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="tbl_conf" displayName="tbl_conf" ref="A1:B11" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="tbl_conf" displayName="tbl_conf" ref="A1:B11" totalsRowShown="0" headerRowDxfId="1">
   <autoFilter ref="A1:B11" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="clé"/>
@@ -1437,20 +1473,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="59" customWidth="1"/>
-    <col min="3" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="19" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="14" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="19" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="14" hidden="1" customWidth="1"/>
     <col min="7" max="9" width="18" customWidth="1"/>
-    <col min="10" max="14" width="14" customWidth="1"/>
-    <col min="15" max="15" width="16.33203125" customWidth="1"/>
-    <col min="16" max="16" width="8.83203125" customWidth="1"/>
+    <col min="10" max="11" width="14" hidden="1" customWidth="1"/>
+    <col min="12" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="16.28515625" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="8.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1497,7 +1535,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>178</v>
       </c>
@@ -1518,12 +1556,11 @@
         <v>0</v>
       </c>
       <c r="M2" s="7">
-        <f>tbl_events[[#This Row],[probability]]</f>
         <v>0.1</v>
       </c>
       <c r="N2" s="7"/>
     </row>
-    <row r="3" spans="1:15" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>45</v>
       </c>
@@ -1539,12 +1576,11 @@
       </c>
       <c r="J3" s="7"/>
       <c r="M3" s="7">
-        <f>specificData!C4</f>
         <v>300</v>
       </c>
       <c r="N3" s="7"/>
     </row>
-    <row r="4" spans="1:15" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>47</v>
       </c>
@@ -1560,12 +1596,11 @@
       </c>
       <c r="J4" s="7"/>
       <c r="M4" s="7">
-        <f>specificData!C5</f>
         <v>1197</v>
       </c>
       <c r="N4" s="7"/>
     </row>
-    <row r="5" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>49</v>
       </c>
@@ -1586,12 +1621,11 @@
         <v>0</v>
       </c>
       <c r="M5" s="7">
-        <f>tbl_events[[#This Row],[probability]]</f>
         <v>1</v>
       </c>
       <c r="N5" s="7"/>
     </row>
-    <row r="6" spans="1:15" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>51</v>
       </c>
@@ -1612,12 +1646,11 @@
         <v>0</v>
       </c>
       <c r="M6" s="7">
-        <f>tbl_events[[#This Row],[probability]]</f>
         <v>1</v>
       </c>
       <c r="N6" s="7"/>
     </row>
-    <row r="7" spans="1:15" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>53</v>
       </c>
@@ -1638,12 +1671,11 @@
         <v>0</v>
       </c>
       <c r="M7" s="7">
-        <f>tbl_events[[#This Row],[probability]]</f>
         <v>3.6299999999999999E-2</v>
       </c>
       <c r="N7" s="7"/>
     </row>
-    <row r="8" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
         <v>28</v>
       </c>
@@ -1654,7 +1686,7 @@
         <v>43</v>
       </c>
       <c r="D8" s="7">
-        <v>4.9999999999999998E-7</v>
+        <v>5.0000000000000004E-6</v>
       </c>
       <c r="G8" s="6">
         <f>IFERROR(VALUE(SUBSTITUTE(tbl_events[[#This Row],[detection_time]],".",","))+VALUE(SUBSTITUTE(tbl_events[[#This Row],[negation_time]],".",",")),0)</f>
@@ -1670,12 +1702,11 @@
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="M8" s="7">
-        <f>tbl_events[[#This Row],[intensity]]</f>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="N8" s="7"/>
     </row>
-    <row r="9" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
         <v>29</v>
       </c>
@@ -1686,7 +1717,7 @@
         <v>43</v>
       </c>
       <c r="D9" s="7">
-        <v>4.9999999999999998E-7</v>
+        <v>5.0000000000000004E-6</v>
       </c>
       <c r="G9" s="6">
         <f>IFERROR(VALUE(SUBSTITUTE(tbl_events[[#This Row],[detection_time]],".",","))+VALUE(SUBSTITUTE(tbl_events[[#This Row],[negation_time]],".",",")),0)</f>
@@ -1699,15 +1730,15 @@
         <v>0</v>
       </c>
       <c r="K9" s="7">
+        <f>tbl_events[[#This Row],[failure_rate]]</f>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="M9" s="7">
-        <f>tbl_events[[#This Row],[intensity]]</f>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="N9" s="7"/>
     </row>
-    <row r="10" spans="1:15" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -1718,8 +1749,7 @@
         <v>43</v>
       </c>
       <c r="D10" s="7">
-        <f>1/(10*8760)</f>
-        <v>1.1415525114155251E-5</v>
+        <v>4.9999999999999998E-7</v>
       </c>
       <c r="G10" s="6">
         <f>IFERROR(VALUE(SUBSTITUTE(tbl_events[[#This Row],[detection_time]],".",","))+VALUE(SUBSTITUTE(tbl_events[[#This Row],[negation_time]],".",",")),0)</f>
@@ -1732,16 +1762,15 @@
         <v>0</v>
       </c>
       <c r="K10" s="7">
-        <f t="shared" ref="K10:K11" si="0">1/(10*8760)</f>
-        <v>1.1415525114155251E-5</v>
+        <f>tbl_events[[#This Row],[failure_rate]]</f>
+        <v>4.9999999999999998E-7</v>
       </c>
       <c r="M10" s="7">
-        <f>tbl_events[[#This Row],[intensity]]</f>
-        <v>1.1415525114155251E-5</v>
+        <v>4.9999999999999998E-7</v>
       </c>
       <c r="N10" s="7"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -1752,8 +1781,7 @@
         <v>43</v>
       </c>
       <c r="D11" s="7">
-        <f>1/(10*8760)</f>
-        <v>1.1415525114155251E-5</v>
+        <v>4.9999999999999998E-7</v>
       </c>
       <c r="G11" s="6">
         <f>IFERROR(VALUE(SUBSTITUTE(tbl_events[[#This Row],[detection_time]],".",","))+VALUE(SUBSTITUTE(tbl_events[[#This Row],[negation_time]],".",",")),0)</f>
@@ -1766,16 +1794,15 @@
         <v>0</v>
       </c>
       <c r="K11" s="7">
-        <f t="shared" si="0"/>
-        <v>1.1415525114155251E-5</v>
+        <f>tbl_events[[#This Row],[failure_rate]]</f>
+        <v>4.9999999999999998E-7</v>
       </c>
       <c r="M11" s="7">
-        <f>tbl_events[[#This Row],[intensity]]</f>
-        <v>1.1415525114155251E-5</v>
+        <v>4.9999999999999998E-7</v>
       </c>
       <c r="N11" s="7"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -1802,12 +1829,11 @@
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="M12" s="7">
-        <f>tbl_events[[#This Row],[intensity]]</f>
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="N12" s="7"/>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -1822,7 +1848,7 @@
       </c>
       <c r="G13" s="6">
         <f>IFERROR(VALUE(SUBSTITUTE(tbl_events[[#This Row],[detection_time]],".",","))+VALUE(SUBSTITUTE(tbl_events[[#This Row],[negation_time]],".",",")),0)</f>
-        <v>2.7777777777777801E-3</v>
+        <v>0</v>
       </c>
       <c r="H13">
         <f>10/3600</f>
@@ -1835,12 +1861,11 @@
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="M13" s="7">
-        <f>tbl_events[[#This Row],[intensity]]</f>
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="N13" s="7"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>161</v>
       </c>
@@ -1872,7 +1897,7 @@
       </c>
       <c r="N14" s="7"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>165</v>
       </c>
@@ -1897,7 +1922,6 @@
         <v>5.0000000000000002E-11</v>
       </c>
       <c r="M15" s="7">
-        <f>tbl_events[[#This Row],[intensity]]</f>
         <v>5.0000000000000002E-11</v>
       </c>
       <c r="N15" s="7"/>
@@ -1920,17 +1944,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:I32"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.5" customWidth="1"/>
-    <col min="2" max="2" width="45.33203125" customWidth="1"/>
-    <col min="3" max="4" width="27.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" customWidth="1"/>
-    <col min="6" max="9" width="15.83203125" customWidth="1"/>
+    <col min="1" max="1" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="45.28515625" customWidth="1"/>
+    <col min="3" max="4" width="27.85546875" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" customWidth="1"/>
+    <col min="6" max="9" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1959,7 +1983,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>5</v>
       </c>
@@ -1978,7 +2002,7 @@
       <c r="H2" s="14"/>
       <c r="I2" s="14"/>
     </row>
-    <row r="3" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>181</v>
       </c>
@@ -1992,7 +2016,7 @@
       <c r="H3" s="14"/>
       <c r="I3" s="14"/>
     </row>
-    <row r="4" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>8</v>
       </c>
@@ -2006,7 +2030,7 @@
       <c r="H4" s="14"/>
       <c r="I4" s="14"/>
     </row>
-    <row r="5" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>10</v>
       </c>
@@ -2020,7 +2044,7 @@
       <c r="H5" s="14"/>
       <c r="I5" s="14"/>
     </row>
-    <row r="6" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>12</v>
       </c>
@@ -2034,7 +2058,7 @@
       <c r="H6" s="14"/>
       <c r="I6" s="14"/>
     </row>
-    <row r="7" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>164</v>
       </c>
@@ -2048,7 +2072,7 @@
       <c r="H7" s="14"/>
       <c r="I7" s="14"/>
     </row>
-    <row r="8" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>15</v>
       </c>
@@ -2065,7 +2089,7 @@
       <c r="H8" s="14"/>
       <c r="I8" s="14"/>
     </row>
-    <row r="9" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>16</v>
       </c>
@@ -2079,7 +2103,7 @@
       <c r="H9" s="14"/>
       <c r="I9" s="14"/>
     </row>
-    <row r="10" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>17</v>
       </c>
@@ -2096,7 +2120,7 @@
       <c r="H10" s="14"/>
       <c r="I10" s="14"/>
     </row>
-    <row r="11" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>19</v>
       </c>
@@ -2110,7 +2134,7 @@
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
     </row>
-    <row r="12" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
         <v>21</v>
       </c>
@@ -2124,7 +2148,7 @@
       <c r="H12" s="14"/>
       <c r="I12" s="14"/>
     </row>
-    <row r="13" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>22</v>
       </c>
@@ -2138,32 +2162,92 @@
       <c r="H13" s="14"/>
       <c r="I13" s="14"/>
     </row>
-    <row r="14" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>24</v>
+        <v>187</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>25</v>
+        <v>186</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
       <c r="F14" s="3"/>
       <c r="G14" s="14"/>
       <c r="H14" s="14"/>
       <c r="I14" s="14"/>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B20" s="7"/>
-    </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B25" s="7"/>
-    </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B28" s="7"/>
+    <row r="15" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="14"/>
+    </row>
+    <row r="16" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+      <c r="I16" s="14"/>
+    </row>
+    <row r="17" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="14"/>
+    </row>
+    <row r="18" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B24" s="7"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B29" s="7"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B32" s="7"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="E2:E502" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="E2:E506" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>BOOL_TF</formula1>
     </dataValidation>
   </dataValidations>
@@ -2176,54 +2260,54 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AN28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:AN34"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" style="3" customWidth="1"/>
-    <col min="2" max="2" width="10.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" style="3" customWidth="1"/>
     <col min="3" max="3" width="25" style="3" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" style="3" customWidth="1"/>
     <col min="5" max="5" width="25" style="3" customWidth="1"/>
-    <col min="6" max="6" width="10.6640625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" style="3" customWidth="1"/>
     <col min="7" max="7" width="25" style="3" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" style="3" customWidth="1"/>
     <col min="9" max="9" width="25" style="3" customWidth="1"/>
-    <col min="10" max="10" width="10.6640625" style="3" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="3" customWidth="1"/>
     <col min="11" max="11" width="25" style="3" customWidth="1"/>
-    <col min="12" max="12" width="10.6640625" style="3" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" style="3" customWidth="1"/>
     <col min="13" max="13" width="25" style="3" customWidth="1"/>
-    <col min="14" max="14" width="10.6640625" style="3" customWidth="1"/>
+    <col min="14" max="14" width="10.7109375" style="3" customWidth="1"/>
     <col min="15" max="15" width="25" style="3" customWidth="1"/>
-    <col min="16" max="16" width="10.6640625" style="3" customWidth="1"/>
+    <col min="16" max="16" width="10.7109375" style="3" customWidth="1"/>
     <col min="17" max="17" width="25" style="3" customWidth="1"/>
-    <col min="18" max="18" width="10.6640625" style="3" customWidth="1"/>
+    <col min="18" max="18" width="10.7109375" style="3" customWidth="1"/>
     <col min="19" max="19" width="25" style="3" customWidth="1"/>
-    <col min="20" max="20" width="10.6640625" style="3" customWidth="1"/>
+    <col min="20" max="20" width="10.7109375" style="3" customWidth="1"/>
     <col min="21" max="21" width="25" style="3" customWidth="1"/>
-    <col min="22" max="22" width="10.6640625" style="3" customWidth="1"/>
+    <col min="22" max="22" width="10.7109375" style="3" customWidth="1"/>
     <col min="23" max="23" width="25" style="3" customWidth="1"/>
-    <col min="24" max="24" width="10.6640625" style="3" customWidth="1"/>
+    <col min="24" max="24" width="10.7109375" style="3" customWidth="1"/>
     <col min="25" max="25" width="25" style="3" customWidth="1"/>
-    <col min="26" max="26" width="10.6640625" style="3" customWidth="1"/>
+    <col min="26" max="26" width="10.7109375" style="3" customWidth="1"/>
     <col min="27" max="27" width="25" style="3" customWidth="1"/>
-    <col min="28" max="28" width="10.6640625" style="3" customWidth="1"/>
+    <col min="28" max="28" width="10.7109375" style="3" customWidth="1"/>
     <col min="29" max="29" width="25" style="3" customWidth="1"/>
-    <col min="30" max="30" width="10.6640625" style="3" customWidth="1"/>
+    <col min="30" max="30" width="10.7109375" style="3" customWidth="1"/>
     <col min="31" max="31" width="25" style="3" customWidth="1"/>
-    <col min="32" max="32" width="10.6640625" style="3" customWidth="1"/>
+    <col min="32" max="32" width="10.7109375" style="3" customWidth="1"/>
     <col min="33" max="33" width="25" style="3" customWidth="1"/>
-    <col min="34" max="34" width="10.6640625" style="3" customWidth="1"/>
+    <col min="34" max="34" width="10.7109375" style="3" customWidth="1"/>
     <col min="35" max="35" width="25" style="3" customWidth="1"/>
-    <col min="36" max="36" width="10.6640625" style="3" customWidth="1"/>
+    <col min="36" max="36" width="10.7109375" style="3" customWidth="1"/>
     <col min="37" max="37" width="25" style="3" customWidth="1"/>
-    <col min="38" max="38" width="10.6640625" style="3" customWidth="1"/>
+    <col min="38" max="38" width="10.7109375" style="3" customWidth="1"/>
     <col min="39" max="39" width="25" style="3" customWidth="1"/>
-    <col min="40" max="40" width="10.6640625" style="3" customWidth="1"/>
-    <col min="41" max="43" width="9.1640625" style="3" customWidth="1"/>
-    <col min="44" max="16384" width="9.1640625" style="3"/>
+    <col min="40" max="40" width="10.7109375" style="3" customWidth="1"/>
+    <col min="41" max="43" width="9.140625" style="3" customWidth="1"/>
+    <col min="44" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>61</v>
       </c>
@@ -2345,7 +2429,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>101</v>
       </c>
@@ -2353,27 +2437,27 @@
         <v>106</v>
       </c>
     </row>
-    <row r="3" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:40" x14ac:dyDescent="0.25">
       <c r="C3" s="3" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="4" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:40" x14ac:dyDescent="0.25">
       <c r="C4" s="3" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="5" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:40" x14ac:dyDescent="0.25">
       <c r="C5" s="3" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="6" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:40" x14ac:dyDescent="0.25">
       <c r="C6" s="3" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="7" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:40" x14ac:dyDescent="0.25">
       <c r="C7" s="3" t="s">
         <v>183</v>
       </c>
@@ -2381,7 +2465,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="8" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:40" x14ac:dyDescent="0.25">
       <c r="E8" s="3" t="s">
         <v>103</v>
       </c>
@@ -2389,12 +2473,12 @@
         <v>106</v>
       </c>
     </row>
-    <row r="9" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:40" x14ac:dyDescent="0.25">
       <c r="G9" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="10" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:40" x14ac:dyDescent="0.25">
       <c r="G10" s="3" t="s">
         <v>105</v>
       </c>
@@ -2402,7 +2486,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:40" x14ac:dyDescent="0.25">
       <c r="I11" s="3" t="s">
         <v>110</v>
       </c>
@@ -2410,7 +2494,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="12" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:40" x14ac:dyDescent="0.25">
       <c r="K12" s="3" t="s">
         <v>111</v>
       </c>
@@ -2418,104 +2502,146 @@
         <v>102</v>
       </c>
     </row>
-    <row r="13" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:40" x14ac:dyDescent="0.25">
       <c r="M13" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="N13" s="3" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:40" x14ac:dyDescent="0.25">
       <c r="O14" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="15" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="O15" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="M16" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="N16" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="O17" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="P14" s="3" t="s">
+      <c r="P17" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="Q18" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="R18" s="3" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="15" spans="1:40" x14ac:dyDescent="0.2">
-      <c r="Q15" s="3" t="s">
+    <row r="19" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="S19" s="3" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="16" spans="1:40" x14ac:dyDescent="0.2">
-      <c r="Q16" s="3" t="s">
+    <row r="20" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="S20" s="3" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="17" spans="5:17" x14ac:dyDescent="0.2">
-      <c r="O17" s="3" t="s">
+    <row r="21" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="Q21" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="R21" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="22" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="S22" s="3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="23" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="O23" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="P17" s="3" t="s">
+      <c r="P23" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="24" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="Q24" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="R24" s="3" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="18" spans="5:17" x14ac:dyDescent="0.2">
-      <c r="Q18" s="3" t="s">
+    <row r="25" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="S25" s="3" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="19" spans="5:17" x14ac:dyDescent="0.2">
-      <c r="Q19" s="3" t="s">
+    <row r="26" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="S26" s="3" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="20" spans="5:17" x14ac:dyDescent="0.2">
-      <c r="M20" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="N20" s="3" t="s">
+    <row r="27" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="Q27" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="R27" s="3" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="21" spans="5:17" x14ac:dyDescent="0.2">
-      <c r="O21" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="22" spans="5:17" x14ac:dyDescent="0.2">
-      <c r="O22" s="3" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="23" spans="5:17" x14ac:dyDescent="0.2">
-      <c r="K23" s="3" t="s">
+    <row r="28" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="S28" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="29" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="K29" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="L23" s="3" t="s">
+      <c r="L29" s="3" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="24" spans="5:17" x14ac:dyDescent="0.2">
-      <c r="M24" s="3" t="s">
+    <row r="30" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="M30" s="3" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="25" spans="5:17" x14ac:dyDescent="0.2">
-      <c r="E25" s="3" t="s">
+    <row r="31" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="E31" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="F31" s="3" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="26" spans="5:17" x14ac:dyDescent="0.2">
-      <c r="G26" s="3" t="s">
+    <row r="32" spans="5:19" x14ac:dyDescent="0.25">
+      <c r="G32" s="3" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="27" spans="5:17" x14ac:dyDescent="0.2">
-      <c r="G27" s="3" t="s">
+    <row r="33" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="G33" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="H27" s="3" t="s">
+      <c r="H33" s="3" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="28" spans="5:17" x14ac:dyDescent="0.2">
-      <c r="I28" s="3" t="s">
+    <row r="34" spans="7:9" x14ac:dyDescent="0.25">
+      <c r="I34" s="3" t="s">
         <v>167</v>
       </c>
     </row>
@@ -2527,10 +2653,10 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valeur invalide" error="Utilisez une valeur autorisée par la liste GATE_TYPES." promptTitle="Type de porte" prompt="Sélectionnez une valeur depuis la liste GATE_TYPES." sqref="Z2 AJ2 AH2 J2 AF2 V2 AD2 L2 F2 AL2 AB2 P2 N2 X2 B2 R2 H2 T2 AN2" xr:uid="{00000000-0002-0000-0200-000003000000}">
       <formula1>GATE_TYPES</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A3:A101 C3:C101 D3:D101 E3:E101 G3:G101 I3:I101 K3:K101 M3:M101 O3:O101 Q3:Q101 S3:S101 U3:U101 W3:W101 Y3:Y101 AA3:AA101 AC3:AC101 AE3:AE101 AG3:AG101 AI3:AI101 AK3:AK101 AM3:AM101" xr:uid="{729B451C-DA96-284D-84B5-7BE46982DBB7}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q3:Q18 Q21:Q24 Q26:Q107 S3:S107 A3:A107 C3:E107 G3:G107 I3:I107 K3:K107 AM3:AM107 U3:U107 W3:W107 Y3:Y107 AA3:AA107 AC3:AC107 AE3:AE107 AG3:AG107 AI3:AI107 AK3:AK107 O3:O107 M3:M107" xr:uid="{729B451C-DA96-284D-84B5-7BE46982DBB7}">
       <formula1>ALL_IDS</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B101 F3:F101 H3:H101 J3:J101 L3:L101 N3:N101 P3:P101 R3:R101 T3:T101 V3:V101 X3:X101 Z3:Z101 AB3:AB101 AD3:AD101 AF3:AF101 AH3:AH101 AJ3:AJ101 AL3:AL101 AN3:AN101" xr:uid="{4CEFD0C8-53F5-AC41-A102-216495CB50A6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B107 F3:F107 H3:H107 J3:J107 L3:L107 AN3:AN107 P3:P107 R3:R107 T3:T107 V3:V107 X3:X107 Z3:Z107 AB3:AB107 AD3:AD107 AF3:AF107 AH3:AH107 AJ3:AJ107 AL3:AL107 N3:N107" xr:uid="{4CEFD0C8-53F5-AC41-A102-216495CB50A6}">
       <formula1>GATE_TYPES</formula1>
     </dataValidation>
   </dataValidations>
@@ -2544,13 +2670,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="46" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>121</v>
       </c>
@@ -2558,7 +2684,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>123</v>
       </c>
@@ -2566,7 +2692,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>125</v>
       </c>
@@ -2574,7 +2700,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>127</v>
       </c>
@@ -2582,7 +2708,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>129</v>
       </c>
@@ -2590,7 +2716,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>130</v>
       </c>
@@ -2598,7 +2724,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>132</v>
       </c>
@@ -2606,7 +2732,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>134</v>
       </c>
@@ -2625,13 +2751,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.5" customWidth="1"/>
-    <col min="2" max="2" width="24.5" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>148</v>
       </c>
@@ -2645,7 +2771,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>185</v>
       </c>
@@ -2660,7 +2786,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>152</v>
       </c>
@@ -2671,7 +2797,7 @@
         <v>1497</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>154</v>
       </c>
@@ -2682,7 +2808,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>156</v>
       </c>
@@ -2694,7 +2820,7 @@
         <v>1197</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>158</v>
       </c>
@@ -2718,18 +2844,18 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="135.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="135.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="77.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="77.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>135</v>
       </c>
@@ -2747,9 +2873,9 @@
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="str" cm="1">
-        <f t="array" ref="A2:A28">_xlfn.VSTACK(tbl_gates[id]&amp;" - "&amp;tbl_gates[label],tbl_events[id]&amp;" - "&amp;tbl_events[label])</f>
+        <f t="array" ref="A2:A32">_xlfn.VSTACK(tbl_gates[id]&amp;" - "&amp;tbl_gates[label],tbl_events[id]&amp;" - "&amp;tbl_events[label])</f>
         <v>COLLISION_ANY_LX - Collision on any LX of the network</v>
       </c>
       <c r="B2" t="s">
@@ -2765,7 +2891,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <v>COLLISION_ANY_LX_SIGNAL_DF - Collision on any LX of the network due to a dangerous failure of a signal (not including other failures such as interlocking, interface to signal…)</v>
       </c>
@@ -2782,7 +2908,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <v>COLLISION_CAT3_NETWORK - Collision on any LX of CAT3 of the network</v>
       </c>
@@ -2796,7 +2922,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <v>COLLISION_CAT12_NETWORK - Collision on any LX of CAT1/CAT2 of the network</v>
       </c>
@@ -2807,7 +2933,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="63.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <v>COLLISION_SPECIFIC_CAT3_LX - Collision on one specific CAT3 LX</v>
       </c>
@@ -2818,7 +2944,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="96" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="96" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <v>COLLISION_SPECIFIC_CAT1_2_LX - Collision on one specific CAT1/CAT2 LX</v>
       </c>
@@ -2827,109 +2953,129 @@
       </c>
       <c r="E7" s="8"/>
     </row>
-    <row r="8" spans="1:6" ht="96" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="96" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <v>DANGEROUS_SIGNALING_ASPECT_CAT3 - DANGEROUS_SIGNALING_ASPECT_CAT3</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <v>NO_RESTRICTIVE_SIGNAL_DISPLAYED - NO_RESTRICTIVE_SIGNAL_DISPLAYED</v>
       </c>
       <c r="E9" s="8"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <v>NO_RESTRICTIVE_SIGNAL_DISPLAYED_LONG_SEQ - No restrictive signal displayed when considering a long sequence to have 2 faulty Uls</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <v>NO_RESTRICTIVE_SIGNAL_DISPLAYED_LOSS_PS - No restrictive signal displayed when considering a loss of PS</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <v>SPURIOUS_PERMISSIVE_SIGNAL_DISPLAYED - SPURIOUS_PERMISSIVE_SIGNAL_DISPLAYED</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <v>DANGEROUS_LOSS_UL1_WITHOUT_ALARM1 - Dangerous loss of UL1 when alarm 1 (barrier) is unavailable</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
+        <v>DANGEROUS_LOSS_ALARM1_WHEN_UL1_DETECTED_FAULTY - Dangerous loss of UL1 when UL1 detected faulty</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="str">
+        <v>UL1_NOT_DETECTED_FAULTY_BY_ITSELF - UL1 not detected faulty by itself and no opening of internal circuit</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="str">
         <v>DANGEROUS_LOSS_UL2_WITHOUT_ALARM2 - Dangerous loss of UL2 when alarm 2 (barrier) is unavailable</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" t="str">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="str">
+        <v>DANGEROUS_LOSS_ALARM2_WHEN_UL2_DETECTED_FAULTY - Dangerous loss of UL2 when UL2 detected faulty</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="str">
+        <v>UL2_NOT_DETECTED_FAULTY_BY_ITSELF - UL2 not detected faulty by itself and no opening of internal circuit</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="str">
         <v>P_LX_CONT - Probability of dangerous failure providing from a signal (and not an Interlocking or interface equipment)</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" t="str">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="str">
         <v>M_CAT3_REP - Multiplicity factor representing the CAT3 LXs by one representative CAT3 LX branch</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" t="str">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="str">
         <v>M_CAT12_REP - Multiplicity factor representing the CAT1/2 LXs by one representative CAT1/2 LX branch</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" t="str">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="str">
         <v>P_TRAIN_PRESENT - Probability of train presence at representative CAT3 LX</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" t="str">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="str">
         <v>P_ROAD_USER_PRESENT - Probability of road user presence at representative CAT3 LX</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" t="str">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="str">
         <v>P_COLLISION_IF_ALL - Probability of collision if all conditions are present</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" t="str">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="str">
         <v>FR_ALARM1 - Dangerous failure of Alarm1 / barrier1</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" t="str">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="str">
         <v>FR_ALARM2 - Dangerous failure of Alarm2 / barrier2</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" t="str">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="str">
         <v>FR_UL1 - Dangerous failure of UL1</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" t="str">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="str">
         <v>FR_UL2 - Dangerous failure of UL2</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" t="str">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="str">
         <v>FR_BIG_ALARM - Dangerous failure of big alarm</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" t="str">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="str">
         <v>FR_PS - Dangerous failure of both PS UL1 and UL2</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" t="str">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="str">
         <v>DF_WHITE_UL_X - Dangerous failure of white UL_X</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" t="str">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="str">
         <v>DF_COLLISION_SPECIFIC_CAT1_2_LX - Dangerous failure leading to collision on CAT1/2 LX</v>
       </c>
     </row>

</xml_diff>